<commit_message>
Update F1 evaluation artifacts
</commit_message>
<xml_diff>
--- a/results/final/figures/table_6_1_retrieval_summary.xlsx
+++ b/results/final/figures/table_6_1_retrieval_summary.xlsx
@@ -473,7 +473,7 @@
         <v>0.286</v>
       </c>
       <c r="F2" t="n">
-        <v>0.223</v>
+        <v>0.235</v>
       </c>
     </row>
     <row r="3">
@@ -490,7 +490,7 @@
         <v>0.304</v>
       </c>
       <c r="F3" t="n">
-        <v>0.193</v>
+        <v>0.206</v>
       </c>
     </row>
     <row r="4">
@@ -507,7 +507,7 @@
         <v>0.327</v>
       </c>
       <c r="F4" t="n">
-        <v>0.182</v>
+        <v>0.193</v>
       </c>
     </row>
     <row r="5">
@@ -524,7 +524,7 @@
         <v>0.354</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2</v>
+        <v>0.216</v>
       </c>
     </row>
     <row r="6">
@@ -541,7 +541,7 @@
         <v>0.354</v>
       </c>
       <c r="F6" t="n">
-        <v>0.181</v>
+        <v>0.194</v>
       </c>
     </row>
     <row r="7">
@@ -558,7 +558,7 @@
         <v>0.366</v>
       </c>
       <c r="F7" t="n">
-        <v>0.185</v>
+        <v>0.196</v>
       </c>
     </row>
     <row r="8">
@@ -575,7 +575,7 @@
         <v>0.366</v>
       </c>
       <c r="F8" t="n">
-        <v>0.172</v>
+        <v>0.181</v>
       </c>
     </row>
     <row r="9">
@@ -592,7 +592,7 @@
         <v>0.375</v>
       </c>
       <c r="F9" t="n">
-        <v>0.169</v>
+        <v>0.178</v>
       </c>
     </row>
     <row r="10">
@@ -609,7 +609,7 @@
         <v>0.375</v>
       </c>
       <c r="F10" t="n">
-        <v>0.154</v>
+        <v>0.161</v>
       </c>
     </row>
     <row r="11">
@@ -626,7 +626,7 @@
         <v>0.379</v>
       </c>
       <c r="F11" t="n">
-        <v>0.146</v>
+        <v>0.153</v>
       </c>
     </row>
     <row r="12">
@@ -648,7 +648,7 @@
         <v>0.207</v>
       </c>
       <c r="F12" t="n">
-        <v>0.149</v>
+        <v>0.157</v>
       </c>
     </row>
     <row r="13">
@@ -665,7 +665,7 @@
         <v>0.293</v>
       </c>
       <c r="F13" t="n">
-        <v>0.22</v>
+        <v>0.233</v>
       </c>
     </row>
     <row r="14">
@@ -682,7 +682,7 @@
         <v>0.316</v>
       </c>
       <c r="F14" t="n">
-        <v>0.203</v>
+        <v>0.214</v>
       </c>
     </row>
     <row r="15">
@@ -699,7 +699,7 @@
         <v>0.342</v>
       </c>
       <c r="F15" t="n">
-        <v>0.202</v>
+        <v>0.214</v>
       </c>
     </row>
     <row r="16">
@@ -716,7 +716,7 @@
         <v>0.349</v>
       </c>
       <c r="F16" t="n">
-        <v>0.193</v>
+        <v>0.203</v>
       </c>
     </row>
     <row r="17">
@@ -733,7 +733,7 @@
         <v>0.355</v>
       </c>
       <c r="F17" t="n">
-        <v>0.185</v>
+        <v>0.194</v>
       </c>
     </row>
     <row r="18">
@@ -750,7 +750,7 @@
         <v>0.355</v>
       </c>
       <c r="F18" t="n">
-        <v>0.164</v>
+        <v>0.171</v>
       </c>
     </row>
     <row r="19">
@@ -767,7 +767,7 @@
         <v>0.355</v>
       </c>
       <c r="F19" t="n">
-        <v>0.154</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="20">
@@ -784,7 +784,7 @@
         <v>0.358</v>
       </c>
       <c r="F20" t="n">
-        <v>0.146</v>
+        <v>0.151</v>
       </c>
     </row>
     <row r="21">
@@ -801,7 +801,7 @@
         <v>0.362</v>
       </c>
       <c r="F21" t="n">
-        <v>0.139</v>
+        <v>0.144</v>
       </c>
     </row>
     <row r="22">
@@ -823,7 +823,7 @@
         <v>0.345</v>
       </c>
       <c r="F22" t="n">
-        <v>0.198</v>
+        <v>0.208</v>
       </c>
     </row>
     <row r="23">
@@ -840,7 +840,7 @@
         <v>0.397</v>
       </c>
       <c r="F23" t="n">
-        <v>0.247</v>
+        <v>0.268</v>
       </c>
     </row>
     <row r="24">
@@ -857,7 +857,7 @@
         <v>0.397</v>
       </c>
       <c r="F24" t="n">
-        <v>0.2</v>
+        <v>0.216</v>
       </c>
     </row>
     <row r="25">
@@ -874,7 +874,7 @@
         <v>0.422</v>
       </c>
       <c r="F25" t="n">
-        <v>0.204</v>
+        <v>0.219</v>
       </c>
     </row>
     <row r="26">
@@ -891,7 +891,7 @@
         <v>0.429</v>
       </c>
       <c r="F26" t="n">
-        <v>0.193</v>
+        <v>0.205</v>
       </c>
     </row>
     <row r="27">
@@ -908,7 +908,7 @@
         <v>0.441</v>
       </c>
       <c r="F27" t="n">
-        <v>0.201</v>
+        <v>0.213</v>
       </c>
     </row>
     <row r="28">
@@ -925,7 +925,7 @@
         <v>0.441</v>
       </c>
       <c r="F28" t="n">
-        <v>0.185</v>
+        <v>0.196</v>
       </c>
     </row>
     <row r="29">
@@ -942,7 +942,7 @@
         <v>0.441</v>
       </c>
       <c r="F29" t="n">
-        <v>0.168</v>
+        <v>0.177</v>
       </c>
     </row>
     <row r="30">
@@ -959,7 +959,7 @@
         <v>0.441</v>
       </c>
       <c r="F30" t="n">
-        <v>0.153</v>
+        <v>0.161</v>
       </c>
     </row>
     <row r="31">
@@ -976,7 +976,7 @@
         <v>0.441</v>
       </c>
       <c r="F31" t="n">
-        <v>0.151</v>
+        <v>0.158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>